<commit_message>
Replaced j:BailBondConditionDescriptionText in BondUpdate with im:ReleaseConditionText in EntityUpdate
</commit_message>
<xml_diff>
--- a/schemas/CaseInitiation_iepd/artifacts/CaseInitiation_MappingSpreasheet.xlsx
+++ b/schemas/CaseInitiation_iepd/artifacts/CaseInitiation_MappingSpreasheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JamesCabral\git\JTMP-Data-Exchange-Specs\schemas\CaseInitiation_iepd\artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76AE029F-FA91-48C7-AA2C-CDC416D5909A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{468A0D4F-5EDB-40AB-AF6D-AE2C09F90C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1857" uniqueCount="982">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1869" uniqueCount="987">
   <si>
     <t/>
   </si>
@@ -3588,6 +3588,21 @@
   <si>
     <t>An identification that references an activity.
 The Item # is the incident number assigned by the Computer Aided Dispatching. It will be included on all arrest paperwork submitted by the arresting officer.</t>
+  </si>
+  <si>
+    <t>A field indicating the condition of the detainees release from custody.</t>
+  </si>
+  <si>
+    <t>ReleaseConditionText</t>
+  </si>
+  <si>
+    <t>im:ReleaseConditionText</t>
+  </si>
+  <si>
+    <t>nola-ext:PersonAugmentationType</t>
+  </si>
+  <si>
+    <t>/nola:CaseInitiationExchange/CourtCase/j:CaseAugmentation/j:CaseDefendantParty/nola-ext:PersonAugmentationType/im:ReleaseConditionText</t>
   </si>
 </sst>
 </file>
@@ -3765,7 +3780,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3844,6 +3859,15 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4353,6 +4377,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Readme"/>
@@ -4433,7 +4458,39 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C1555FB-E16C-423D-A1FA-98AD99C9E15B}" name="MappingSpreadsheet" displayName="MappingSpreadsheet" ref="A1:N146" totalsRowShown="0" headerRowDxfId="18" dataDxfId="16" headerRowBorderDxfId="17" tableBorderDxfId="15" totalsRowBorderDxfId="14">
-  <autoFilter ref="A1:N146" xr:uid="{2C1555FB-E16C-423D-A1FA-98AD99C9E15B}"/>
+  <autoFilter xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" ref="A1:N146" xr:uid="{2C1555FB-E16C-423D-A1FA-98AD99C9E15B}">
+    <filterColumn colId="12">
+      <filters>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <x14:filter val="/CourtCase/j:CaseAugmentation/j:CaseDefendantQuantityText"/>
+            <x14:filter val="/j:BookingSubject/RoleOfPerson/nola-ext:PersonAugmentation/nola-ext:CaseDefendantNumber_x000a_/j:CourtOrderDesignatedSubject/RoleOfPerson/nola-ext:PersonAugmentation/nola-ext:CaseDefendantNumber_x000a_/j:CaseDefendantParty/EntityPerson/nola-ext:PersonAugmentation/nola-ext:CaseDefendantNumber"/>
+            <x14:filter val="/j:CaseDefendantParty/EntityPerson/PersonDescriptionText"/>
+            <x14:filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonBirthDate/nc:DateRepresentation/nc:Date"/>
+            <x14:filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonName/nc:MiddleName_x000a_/Person/PersonName/PersonMiddleName"/>
+            <x14:filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonName/nc:PersonFullName"/>
+            <x14:filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonName/nc:PersonGivenName_x000a__x000a_/nc:RoleOfPerson/nc:PersonName/nc:GivenName"/>
+            <x14:filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonName/nc:PersonSurName"/>
+            <x14:filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonName/PersonNameSuffixText"/>
+            <x14:filter val="/nola:CaseInitiationExchange/CourtCase/j:CaseAugmentation/j:CaseDefendantParty/nola-ext:DefendantAugmentationType/nola-ext:InmateDefendant_x000a_"/>
+            <x14:filter val="/Person/PersonSSNIdentification/IdentificationID_x000a_/j:CaseDefendantParty/EntityPerson/PersonSSNIdentification/IdentificationID"/>
+          </mc:Choice>
+          <mc:Fallback>
+            <filter val="/CourtCase/j:CaseAugmentation/j:CaseDefendantQuantityText"/>
+            <filter val="/j:CaseDefendantParty/EntityPerson/PersonDescriptionText"/>
+            <filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonBirthDate/nc:DateRepresentation/nc:Date"/>
+            <filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonName/nc:MiddleName_x000a_/Person/PersonName/PersonMiddleName"/>
+            <filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonName/nc:PersonFullName"/>
+            <filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonName/nc:PersonGivenName_x000a__x000a_/nc:RoleOfPerson/nc:PersonName/nc:GivenName"/>
+            <filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonName/nc:PersonSurName"/>
+            <filter val="/nc:CourtCase/nc:CaseAugmentationPoint/j:CaseAugmentation/j:CaseDefendantParty/nc:EntityPerson/nc:PersonName/PersonNameSuffixText"/>
+            <filter val="/nola:CaseInitiationExchange/CourtCase/j:CaseAugmentation/j:CaseDefendantParty/nola-ext:DefendantAugmentationType/nola-ext:InmateDefendant_x000a_"/>
+            <filter val="/Person/PersonSSNIdentification/IdentificationID_x000a_/j:CaseDefendantParty/EntityPerson/PersonSSNIdentification/IdentificationID"/>
+          </mc:Fallback>
+        </mc:AlternateContent>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{A154B48A-3186-466D-92F1-8A6270997FD4}" name="Property Type" dataDxfId="13"/>
     <tableColumn id="2" xr3:uid="{34D42627-CEA6-4CC6-8595-04D65F5B7FC2}" name="ID" dataDxfId="12"/>
@@ -4751,7 +4808,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P158"/>
+  <dimension ref="A1:P159"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15.46484375" customWidth="1"/>
@@ -4812,7 +4869,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -4840,7 +4897,7 @@
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
     </row>
-    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
@@ -4882,7 +4939,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
@@ -4924,7 +4981,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="7" t="s">
         <v>12</v>
       </c>
@@ -4966,7 +5023,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="7" t="s">
         <v>12</v>
       </c>
@@ -5008,7 +5065,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="7" t="s">
         <v>12</v>
       </c>
@@ -5050,7 +5107,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
@@ -5080,7 +5137,7 @@
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
     </row>
-    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="7" t="s">
         <v>12</v>
       </c>
@@ -5122,7 +5179,7 @@
         <v>836</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="7" t="s">
         <v>12</v>
       </c>
@@ -5164,7 +5221,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
@@ -5194,7 +5251,7 @@
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
     </row>
-    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="7" t="s">
         <v>12</v>
       </c>
@@ -5236,7 +5293,7 @@
         <v>838</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>8</v>
       </c>
@@ -5266,7 +5323,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="7" t="s">
         <v>12</v>
       </c>
@@ -5308,7 +5365,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="7" t="s">
         <v>12</v>
       </c>
@@ -5350,7 +5407,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="7" t="s">
         <v>12</v>
       </c>
@@ -5392,7 +5449,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="7" t="s">
         <v>12</v>
       </c>
@@ -5434,7 +5491,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="7" t="s">
         <v>12</v>
       </c>
@@ -5476,7 +5533,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="7" t="s">
         <v>12</v>
       </c>
@@ -5518,7 +5575,7 @@
         <v>845</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="7" t="s">
         <v>12</v>
       </c>
@@ -5560,7 +5617,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="7" t="s">
         <v>12</v>
       </c>
@@ -5602,7 +5659,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="7" t="s">
         <v>12</v>
       </c>
@@ -5644,7 +5701,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="7" t="s">
         <v>12</v>
       </c>
@@ -5686,7 +5743,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="3" t="s">
         <v>8</v>
       </c>
@@ -5714,7 +5771,7 @@
       <c r="M24" s="4"/>
       <c r="N24" s="4"/>
     </row>
-    <row r="25" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="11" t="s">
         <v>410</v>
       </c>
@@ -5750,7 +5807,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="7" t="s">
         <v>12</v>
       </c>
@@ -5792,7 +5849,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="7" t="s">
         <v>12</v>
       </c>
@@ -5834,7 +5891,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="3" t="s">
         <v>8</v>
       </c>
@@ -5862,7 +5919,7 @@
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
     </row>
-    <row r="29" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="3" t="s">
         <v>8</v>
       </c>
@@ -5890,7 +5947,7 @@
       <c r="M29" s="4"/>
       <c r="N29" s="4"/>
     </row>
-    <row r="30" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="7" t="s">
         <v>12</v>
       </c>
@@ -5932,7 +5989,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="7" t="s">
         <v>12</v>
       </c>
@@ -5974,7 +6031,7 @@
         <v>854</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="11" t="s">
         <v>410</v>
       </c>
@@ -6012,7 +6069,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="11" t="s">
         <v>410</v>
       </c>
@@ -6052,7 +6109,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="7" t="s">
         <v>12</v>
       </c>
@@ -6094,7 +6151,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="7" t="s">
         <v>12</v>
       </c>
@@ -6134,7 +6191,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="7" t="s">
         <v>12</v>
       </c>
@@ -6176,7 +6233,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="7" t="s">
         <v>12</v>
       </c>
@@ -6220,7 +6277,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="7" t="s">
         <v>12</v>
       </c>
@@ -6264,7 +6321,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="7" t="s">
         <v>12</v>
       </c>
@@ -6306,7 +6363,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="7" t="s">
         <v>12</v>
       </c>
@@ -6348,7 +6405,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="7" t="s">
         <v>12</v>
       </c>
@@ -6390,7 +6447,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="7" t="s">
         <v>12</v>
       </c>
@@ -6432,7 +6489,7 @@
         <v>865</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="7" t="s">
         <v>12</v>
       </c>
@@ -6474,7 +6531,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="7" t="s">
         <v>12</v>
       </c>
@@ -6518,7 +6575,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="11" t="s">
         <v>410</v>
       </c>
@@ -6558,7 +6615,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="7" t="s">
         <v>12</v>
       </c>
@@ -6600,7 +6657,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="7" t="s">
         <v>12</v>
       </c>
@@ -6642,7 +6699,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="7" t="s">
         <v>12</v>
       </c>
@@ -6686,7 +6743,7 @@
         <v>871</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="7" t="s">
         <v>12</v>
       </c>
@@ -6730,7 +6787,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="3" t="s">
         <v>8</v>
       </c>
@@ -6764,7 +6821,7 @@
       </c>
       <c r="N50" s="4"/>
     </row>
-    <row r="51" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="7" t="s">
         <v>12</v>
       </c>
@@ -6806,7 +6863,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="7" t="s">
         <v>12</v>
       </c>
@@ -6848,7 +6905,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" s="7" t="s">
         <v>12</v>
       </c>
@@ -6890,7 +6947,7 @@
         <v>875</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="11" t="s">
         <v>410</v>
       </c>
@@ -6926,7 +6983,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="7" t="s">
         <v>12</v>
       </c>
@@ -6970,7 +7027,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="7" t="s">
         <v>12</v>
       </c>
@@ -7014,7 +7071,7 @@
         <v>878</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" s="7" t="s">
         <v>12</v>
       </c>
@@ -7058,7 +7115,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="7" t="s">
         <v>12</v>
       </c>
@@ -7100,7 +7157,7 @@
         <v>880</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="7" t="s">
         <v>12</v>
       </c>
@@ -7142,7 +7199,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="60" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="3" t="s">
         <v>8</v>
       </c>
@@ -7178,7 +7235,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A61" s="11" t="s">
         <v>410</v>
       </c>
@@ -7212,7 +7269,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="7" t="s">
         <v>12</v>
       </c>
@@ -7296,7 +7353,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="64" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="7" t="s">
         <v>12</v>
       </c>
@@ -7338,7 +7395,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="65" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A65" s="11" t="s">
         <v>410</v>
       </c>
@@ -7378,7 +7435,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="66" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A66" s="7" t="s">
         <v>12</v>
       </c>
@@ -7422,7 +7479,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="67" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A67" s="11" t="s">
         <v>410</v>
       </c>
@@ -7458,7 +7515,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="68" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" s="7" t="s">
         <v>12</v>
       </c>
@@ -7502,7 +7559,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" s="7" t="s">
         <v>12</v>
       </c>
@@ -7544,7 +7601,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A70" s="7" t="s">
         <v>12</v>
       </c>
@@ -7588,7 +7645,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="11" t="s">
         <v>410</v>
       </c>
@@ -7626,7 +7683,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A72" s="7" t="s">
         <v>12</v>
       </c>
@@ -7668,7 +7725,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="7" t="s">
         <v>12</v>
       </c>
@@ -7710,7 +7767,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A74" s="11" t="s">
         <v>410</v>
       </c>
@@ -7746,7 +7803,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="75" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A75" s="7" t="s">
         <v>12</v>
       </c>
@@ -7782,7 +7839,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="76" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A76" s="7" t="s">
         <v>12</v>
       </c>
@@ -7818,7 +7875,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="77" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A77" s="7" t="s">
         <v>12</v>
       </c>
@@ -7860,7 +7917,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="78" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A78" s="7" t="s">
         <v>12</v>
       </c>
@@ -7900,7 +7957,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="79" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A79" s="7" t="s">
         <v>12</v>
       </c>
@@ -7936,7 +7993,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="80" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A80" s="3" t="s">
         <v>8</v>
       </c>
@@ -7968,7 +8025,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="81" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A81" s="7" t="s">
         <v>12</v>
       </c>
@@ -8010,7 +8067,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="82" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A82" s="3" t="s">
         <v>8</v>
       </c>
@@ -8046,7 +8103,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="83" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A83" s="7" t="s">
         <v>12</v>
       </c>
@@ -8090,7 +8147,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="84" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A84" s="7" t="s">
         <v>12</v>
       </c>
@@ -8132,7 +8189,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="85" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A85" s="7" t="s">
         <v>12</v>
       </c>
@@ -8174,7 +8231,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="86" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A86" s="7" t="s">
         <v>12</v>
       </c>
@@ -8216,7 +8273,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="87" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A87" s="3" t="s">
         <v>8</v>
       </c>
@@ -8250,7 +8307,7 @@
       </c>
       <c r="N87" s="4"/>
     </row>
-    <row r="88" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A88" s="7" t="s">
         <v>12</v>
       </c>
@@ -8292,7 +8349,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="89" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A89" s="7" t="s">
         <v>12</v>
       </c>
@@ -8334,7 +8391,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="90" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A90" s="7" t="s">
         <v>12</v>
       </c>
@@ -8378,7 +8435,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="91" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A91" s="7" t="s">
         <v>12</v>
       </c>
@@ -8422,7 +8479,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="92" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A92" s="11" t="s">
         <v>410</v>
       </c>
@@ -8460,7 +8517,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="93" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A93" s="3" t="s">
         <v>8</v>
       </c>
@@ -8576,7 +8633,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="96" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A96" s="11" t="s">
         <v>410</v>
       </c>
@@ -8616,7 +8673,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="97" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A97" s="3" t="s">
         <v>8</v>
       </c>
@@ -8644,7 +8701,7 @@
       <c r="M97" s="4"/>
       <c r="N97" s="4"/>
     </row>
-    <row r="98" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A98" s="7" t="s">
         <v>12</v>
       </c>
@@ -8686,7 +8743,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="99" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A99" s="7" t="s">
         <v>12</v>
       </c>
@@ -8728,7 +8785,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="100" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A100" s="3" t="s">
         <v>8</v>
       </c>
@@ -8760,7 +8817,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="101" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A101" s="3" t="s">
         <v>8</v>
       </c>
@@ -8790,7 +8847,7 @@
       <c r="M101" s="4"/>
       <c r="N101" s="4"/>
     </row>
-    <row r="102" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A102" s="7" t="s">
         <v>12</v>
       </c>
@@ -8832,7 +8889,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="103" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A103" s="7" t="s">
         <v>12</v>
       </c>
@@ -8874,7 +8931,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="104" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A104" s="3" t="s">
         <v>8</v>
       </c>
@@ -8908,7 +8965,7 @@
       </c>
       <c r="N104" s="4"/>
     </row>
-    <row r="105" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A105" s="3" t="s">
         <v>8</v>
       </c>
@@ -8938,7 +8995,7 @@
       </c>
       <c r="N105" s="4"/>
     </row>
-    <row r="106" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A106" s="7" t="s">
         <v>12</v>
       </c>
@@ -8980,7 +9037,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="107" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A107" s="7" t="s">
         <v>12</v>
       </c>
@@ -9022,7 +9079,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="108" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A108" s="7" t="s">
         <v>12</v>
       </c>
@@ -9064,7 +9121,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="109" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A109" s="7" t="s">
         <v>12</v>
       </c>
@@ -9106,7 +9163,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="110" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A110" s="3" t="s">
         <v>8</v>
       </c>
@@ -9136,7 +9193,7 @@
       <c r="M110" s="4"/>
       <c r="N110" s="4"/>
     </row>
-    <row r="111" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A111" s="3" t="s">
         <v>8</v>
       </c>
@@ -9166,7 +9223,7 @@
       <c r="M111" s="4"/>
       <c r="N111" s="4"/>
     </row>
-    <row r="112" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A112" s="7" t="s">
         <v>12</v>
       </c>
@@ -9208,7 +9265,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="113" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A113" s="3" t="s">
         <v>8</v>
       </c>
@@ -9234,7 +9291,7 @@
       <c r="M113" s="4"/>
       <c r="N113" s="4"/>
     </row>
-    <row r="114" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A114" s="7" t="s">
         <v>12</v>
       </c>
@@ -9274,7 +9331,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="115" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A115" s="7" t="s">
         <v>12</v>
       </c>
@@ -9316,7 +9373,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="116" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A116" s="7" t="s">
         <v>12</v>
       </c>
@@ -9358,7 +9415,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="117" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A117" s="3" t="s">
         <v>8</v>
       </c>
@@ -9386,7 +9443,7 @@
       <c r="M117" s="4"/>
       <c r="N117" s="4"/>
     </row>
-    <row r="118" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A118" s="11" t="s">
         <v>410</v>
       </c>
@@ -9426,7 +9483,7 @@
         <v>928</v>
       </c>
     </row>
-    <row r="119" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A119" s="11" t="s">
         <v>410</v>
       </c>
@@ -9466,7 +9523,7 @@
         <v>928</v>
       </c>
     </row>
-    <row r="120" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A120" s="11" t="s">
         <v>410</v>
       </c>
@@ -9506,7 +9563,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="121" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A121" s="3" t="s">
         <v>8</v>
       </c>
@@ -9534,7 +9591,7 @@
       <c r="M121" s="4"/>
       <c r="N121" s="4"/>
     </row>
-    <row r="122" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A122" s="7" t="s">
         <v>12</v>
       </c>
@@ -9576,7 +9633,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="123" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A123" s="7" t="s">
         <v>12</v>
       </c>
@@ -9618,7 +9675,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="124" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A124" s="7" t="s">
         <v>12</v>
       </c>
@@ -9660,7 +9717,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="125" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A125" s="3" t="s">
         <v>8</v>
       </c>
@@ -9770,7 +9827,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="128" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A128" s="7" t="s">
         <v>12</v>
       </c>
@@ -9854,7 +9911,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="130" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A130" s="3" t="s">
         <v>8</v>
       </c>
@@ -10098,7 +10155,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="136" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A136" s="3" t="s">
         <v>8</v>
       </c>
@@ -10126,7 +10183,7 @@
       <c r="M136" s="4"/>
       <c r="N136" s="4"/>
     </row>
-    <row r="137" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A137" s="7" t="s">
         <v>12</v>
       </c>
@@ -10168,7 +10225,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="138" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A138" s="7" t="s">
         <v>12</v>
       </c>
@@ -10210,7 +10267,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="139" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A139" s="7" t="s">
         <v>12</v>
       </c>
@@ -10252,7 +10309,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="140" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A140" s="7" t="s">
         <v>12</v>
       </c>
@@ -10294,7 +10351,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="141" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="141" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A141" s="7" t="s">
         <v>12</v>
       </c>
@@ -10336,7 +10393,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="142" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="142" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A142" s="3" t="s">
         <v>8</v>
       </c>
@@ -10366,7 +10423,7 @@
       <c r="M142" s="4"/>
       <c r="N142" s="4"/>
     </row>
-    <row r="143" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A143" s="7" t="s">
         <v>12</v>
       </c>
@@ -10408,7 +10465,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="144" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A144" s="3" t="s">
         <v>8</v>
       </c>
@@ -10438,7 +10495,7 @@
       <c r="M144" s="4"/>
       <c r="N144" s="4"/>
     </row>
-    <row r="145" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A145" s="7" t="s">
         <v>12</v>
       </c>
@@ -10480,7 +10537,7 @@
         <v>948</v>
       </c>
     </row>
-    <row r="146" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A146" s="7" t="s">
         <v>12</v>
       </c>
@@ -11024,6 +11081,46 @@
       </c>
       <c r="O158" s="25"/>
       <c r="P158" s="25"/>
+    </row>
+    <row r="159" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A159" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="B159" s="16"/>
+      <c r="C159" s="29" t="s">
+        <v>408</v>
+      </c>
+      <c r="D159" s="29" t="s">
+        <v>983</v>
+      </c>
+      <c r="E159" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F159" s="30" t="s">
+        <v>982</v>
+      </c>
+      <c r="G159" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="H159" s="29" t="s">
+        <v>983</v>
+      </c>
+      <c r="I159" s="16"/>
+      <c r="J159" s="16" t="s">
+        <v>984</v>
+      </c>
+      <c r="K159" s="21" t="s">
+        <v>460</v>
+      </c>
+      <c r="L159" s="16" t="s">
+        <v>985</v>
+      </c>
+      <c r="M159" s="16" t="s">
+        <v>986</v>
+      </c>
+      <c r="N159" s="16" t="s">
+        <v>986</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O147">
@@ -11036,10 +11133,13 @@
       <formula1>MAPPING_CODES</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="J159" r:id="rId1" xr:uid="{BB734526-8C28-4539-863E-8008359E5F93}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>